<commit_message>
feature: finish 2 function update_student_lms and report_lms
</commit_message>
<xml_diff>
--- a/data/output/report_perform_lms/252/__danh_sach_khong_thuc_hien_lms.xlsx
+++ b/data/output/report_perform_lms/252/__danh_sach_khong_thuc_hien_lms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -777,6 +777,58 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>06-04-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Luật</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TB110</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BLAW2303</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Luật lao động</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TB124342,TB224342</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Trung tâm Chính trị phường Tân Hòa</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KI211</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Trần Thị Kim Huế</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>13-04-2026</t>
         </is>
       </c>
     </row>

</xml_diff>